<commit_message>
refactor: update triplet extraction, embedding, and query flow logic while synchronizing associated output datasets
</commit_message>
<xml_diff>
--- a/src/Query/output/batch_result.xlsx
+++ b/src/Query/output/batch_result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranhuuduc/Documents/dev/Rag_Graph_LawLaw/src/Query/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F64AC0-487F-9445-853F-84DF64F3B251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DA0D9B-4258-F142-A0D5-C4723096B530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1280" yWindow="-18960" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="191">
   <si>
     <t>Câu hỏi</t>
   </si>
@@ -348,6 +348,388 @@
 2. Phạt tiền từ 6.000.000 đồng đến 8.000.000 đồng nếu nồng độ cồn trong máu hoặc hơi thở vượt quá 50 miligam đến 80 miligam/100 mililít máu hoặc vượt quá 0,25 miligam đến 0,4 miligam/1 lít khí thở (Điều 7, Khoản 8, Điểm b - Nghị định 168:2024/NĐ-CP).
 3. Phạt tiền từ 8.000.000 đồng đến 10.000.000 đồng nếu nồng độ cồn trong máu hoặc hơi thở vượt quá 80 miligam/100 mililít máu hoặc vượt quá 0,4 miligam/1 lít khí thở (Điều 7, Khoản 9, Điểm d - Nghị định 168:2024/NĐ-CP).
 Vì vậy, nếu mức phạt của bạn là hơn 15 triệu đồng, có thể có các yếu tố khác hoặc vi phạm khác không được liệt kê trong các điều khoản này.</t>
+  </si>
+  <si>
+    <t>Vượt đèn đỏ mém tung ngta có phạt nặng k mọi người</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời câu hỏi này. Không có điều khoản nào trong danh sách cung cấp đề cập đến việc vượt đèn đỏ hoặc mức phạt cụ thể cho hành vi này.</t>
+  </si>
+  <si>
+    <t>mọi người cho mình hỏi, mình bị phạt ở ngay hầm thủ thiêm hơn 2 năm rồi, đã mất giấy phạt, bị thu bằng. vậy bây giờ ra đâu nộp phạt và mất giấy rồi thì nộp phạt có được không ạ</t>
+  </si>
+  <si>
+    <t>Xe mua cũ lâu rồi lúc mua chỉ viết giấy tay , có cavet xe nhưng người khác đứng tên vs mất liên lạc chủ củ , nay em bị vphc giam xe có nộp phạt được lấy xe được không ạ , hay phải cần có cccd chủ củ</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời câu hỏi về việc bạn có thể nộp phạt để lấy lại xe khi bị vi phạm hành chính mà không có giấy tờ chính chủ hay không.</t>
+  </si>
+  <si>
+    <t>em có bị phạt do chở người k đội mũ. Em có đóng phạt trên dichvucong r mà vẫn chưa thấy gửi giấy dky xe về nên em gọi thì ngta bảo bạn đi cùng cũng phải đóng phạt nma bạn ý bảo k thấy trên dichvucong thì không biết phải nộp phạt thế nào ạ. Mà em thấy họ bảo mỗi chỗ phải đóng phạt khác nhau, bạn ý ở Bắc Ninh thì phải đóng bao nhiêu ạ.</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, nếu bạn chở người không đội mũ bảo hiểm hoặc đội mũ bảo hiểm không cài quai đúng quy cách, bạn có thể bị phạt tiền từ 400.000 đồng đến 600.000 đồng (Điều 7, Khoản 2, Điểm h - Nghị định 168:2024/NĐ-CP).
+Về việc người đi cùng bạn cũng phải đóng phạt, điều khoản không đề cập cụ thể về việc xử phạt người ngồi sau không đội mũ bảo hiểm. Tuy nhiên, nếu người đi cùng bạn là người điều khiển xe đạp máy và không đội mũ bảo hiểm, họ có thể bị phạt từ 400.000 đồng đến 600.000 đồng (Điều 9, Khoản 4, Điểm d - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử phạt cụ thể cho người ngồi sau trên xe mô tô, xe máy không đội mũ bảo hiểm, cũng như không có thông tin về việc xử phạt khác nhau theo địa phương. Do đó, bạn nên liên hệ với cơ quan chức năng tại địa phương để biết thêm chi tiết về việc nộp phạt và các thủ tục liên quan.</t>
+  </si>
+  <si>
+    <t>Các bác cho em hỏi trc e bị sử phạt ở xã cũ chưa xác nhập bị mất tờ giấy quyết định rồi giờ muốn nộp online lại k đc còn cách nào k ạ</t>
+  </si>
+  <si>
+    <t>T9/2019 em bị xử lý vi phạm và đã đóng phạt vào T11/2019 mà bây giờ lại hiện lỗi vẫn còn treo. Mà em bị ở cam ranh,trong khi đó em đang ở sài gòn. Thì có cách nào giải quyết nhanh chóng ko ạ. Em cảm ơn!</t>
+  </si>
+  <si>
+    <t>AC cho e hỏi 1 chút. E bị phạt k gương tay trái từ ngày 30/4 đến ngày 09/5 đã lên nộp phạt có biên thu của ngân hàng. Nhưng mà hôm nay ngày 25/11 lại có tin nhắn quyết định xử phạt ạ. AC cho e xin ý kiến xử lý thế nào ạ</t>
+  </si>
+  <si>
+    <t>Các điều khoản không đề cập tới việc xử lý tình huống khi đã nộp phạt nhưng vẫn nhận được tin nhắn quyết định xử phạt sau đó. Tuy nhiên, theo điều khoản cung cấp, hành vi điều khiển xe không có gương chiếu hậu bên trái có thể bị phạt tiền từ 400.000 đồng đến 600.000 đồng (Điều 14, Khoản 1, Điểm a - Nghị định 168:2024/NĐ-CP). 
+Để giải quyết tình huống này, bạn nên liên hệ với cơ quan đã ra quyết định xử phạt để xác minh và cung cấp bằng chứng về việc đã nộp phạt trước đó.</t>
+  </si>
+  <si>
+    <t>Ae cho hỏi camera AI có quét vị phạm ko gương ko ạ</t>
+  </si>
+  <si>
+    <t>Các điều khoản không đề cập tới việc camera AI có thể quét và phát hiện vi phạm không có gương chiếu hậu. Tuy nhiên, điều khoản có nêu rằng việc điều khiển xe không có đủ gương chiếu hậu có thể bị phạt tiền từ 400.000 đồng đến 600.000 đồng (Điều 13, Khoản 2, Điểm a - Nghị định 168:2024/NĐ-CP).</t>
+  </si>
+  <si>
+    <t>Xin chia sẻ chút kinh nghiệm
+- e bị phạt k mũ ( quá hạn 1 năm ) ( ở xuân la-hà nội )
+- giờ e muốn đóng phạt online ( e bị mất giấy phạt rồi,có cách nào kiểm tra và đóng phạt kạ )</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được chỉ đề cập đến mức phạt tiền đối với hành vi không đội mũ bảo hiểm khi điều khiển xe mô tô, xe máy hoặc xe đạp máy, với mức phạt từ 400.000 đồng đến 600.000 đồng (Điều 7, Khoản 2, Điểm h - Nghị định 168:2024/NĐ-CP; Điều 9, Khoản 4, Điểm d - Nghị định 168:2024/NĐ-CP).
+Tuy nhiên, các điều khoản không đề cập tới việc kiểm tra và đóng phạt online, cũng như không cung cấp thông tin về cách xử lý khi mất giấy phạt.</t>
+  </si>
+  <si>
+    <t>Mọi người cho e hỏi lỗi đi ngược chiều bị lập biên bản tước bằng lái xe, khi đóng phạt mình đóng khoản bao nhiêu ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, nếu bạn bị lập biên bản vì lỗi đi ngược chiều, mức phạt tiền sẽ phụ thuộc vào loại đường mà bạn vi phạm:
+1. Nếu bạn đi ngược chiều trên đường một chiều hoặc trên đường có biển “Cấm đi ngược chiều”, mức phạt tiền từ 18.000.000 đồng đến 20.000.000 đồng (Điều 6, Khoản 9, Điểm d - Nghị định 168:2024/NĐ-CP).
+2. Nếu bạn đi ngược chiều trên đường cao tốc, mức phạt tiền từ 30.000.000 đồng đến 40.000.000 đồng (Điều 6, Khoản 11, Điểm đ - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc tước bằng lái xe trong trường hợp này.</t>
+  </si>
+  <si>
+    <t>Em giao xe cho bạn đi tháo biển kiểm soát không bằng lái, gương chiếu hậu bên trái. Các bác cho em hỏi có hết nhiều không ạ…</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, việc giao xe cho bạn đi mà không có giấy phép lái xe và không có gương chiếu hậu bên trái có thể dẫn đến các mức phạt sau:
+1. **Không có giấy phép lái xe**: 
+   - Phạt tiền từ 2.000.000 đồng đến 4.000.000 đồng đối với người điều khiển xe mô tô hai bánh có dung tích xi-lanh đến 125 cm3 hoặc có công suất động cơ điện đến 11 kW nếu không có giấy phép lái xe (Điều 18, Khoản 5, Điểm a - Nghị định 168:2024/NĐ-CP).
+2. **Không có gương chiếu hậu bên trái**:
+   - Phạt tiền từ 400.000 đồng đến 600.000 đồng đối với hành vi điều khiển xe không có gương chiếu hậu bên trái người điều khiển hoặc có nhưng không có tác dụng (Điều 14, Khoản 1, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc tháo biển kiểm soát.</t>
+  </si>
+  <si>
+    <t>Ae cho hỏi tí xe tên của mẹ m m bị bắt lỗi k bằng với k gương thì phạt tầm bao nhiêu nhỉ (150cc)</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc điều khiển xe mô tô không có gương chiếu hậu bên trái hoặc có nhưng không có tác dụng sẽ bị phạt tiền từ 400.000 đồng đến 600.000 đồng (Điều 14, Khoản 1, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử phạt khi không có bằng lái xe cho xe có dung tích xi-lanh 150cc.</t>
+  </si>
+  <si>
+    <t>Mọi người ơi cho e hỏi cho bạn mượn xe gây tai nạn thì phạt người giao xe với người k bằng là bao nhiêu ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc cho bạn mượn xe gây tai nạn có thể liên quan đến hai đối tượng: người giao xe và người điều khiển xe.
+1. **Người giao xe**: 
+   - Giao xe cơ giới cho người không đủ điều kiện điều khiển xe tham gia giao thông là hành vi bị nghiêm cấm (Điều 9, Khoản 7 - Luật số: 36/2024/QH15). Tuy nhiên, các điều khoản không đề cập cụ thể mức phạt cho người giao xe trong trường hợp này.
+2. **Người điều khiển xe**:
+   - Nếu người điều khiển xe gây tai nạn giao thông và không dừng ngay phương tiện, không giữ nguyên hiện trường, không trợ giúp người bị nạn, không ở lại hiện trường hoặc không đến trình báo ngay với cơ quan công an, mức phạt là từ 16.000.000 đồng đến 18.000.000 đồng (Điều 6, Khoản 8 - Nghị định 168:2024/NĐ-CP).
+   - Nếu người điều khiển xe thực hiện các hành vi vi phạm như không quan sát, không giảm tốc độ, không đi đúng phần đường, làn đường, hoặc các hành vi khác gây tai nạn giao thông, mức phạt là từ 20.000.000 đồng đến 22.000.000 đồng (Điều 6, Khoản 10, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử phạt cụ thể đối với người giao xe trong trường hợp này.</t>
+  </si>
+  <si>
+    <t>Xe mua lâu rồi bị bắt không chính chủ , giờ lên phạt cs kêu mang cccd chủ cũ mà giờ không tìm được chủ củ phải giải quyết như nào mới được phạt AE</t>
+  </si>
+  <si>
+    <t>Chủ phương tiện SH này chuyển hướng vào quán trà đá vỉa hè không có tín hiệu, người điều khiển phương tiện không đội mũ bảo hiểm và gây tai nạn, trốn tránh, không giúp đỡ hay xin lỗi mà còn chửi lại người bị ngã tại Ngã Tư Lương Thế Vinh - Tố Hữu địa bàn quận Thanh Xuân, Hà Nội vào thời điểm 8h20p đến 8h35p ngày 14/11/2025. Rất mong các lực lượng check cam và phạt nguội thật nặng với trường hợp này.</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, người điều khiển xe SH đã vi phạm các quy định sau:
+1. **Chuyển hướng không có tín hiệu**: Người điều khiển xe SH chuyển hướng vào quán trà đá mà không có tín hiệu báo trước, vi phạm quy định về chuyển hướng (Điều 7, Khoản 3, Điểm a - Nghị định 168:2024/NĐ-CP). Mức phạt cho hành vi này là từ 600.000 đồng đến 800.000 đồng.
+2. **Không đội mũ bảo hiểm**: Người điều khiển xe không đội mũ bảo hiểm khi tham gia giao thông, vi phạm quy định về đội mũ bảo hiểm (Điều 7, Khoản 2, Điểm h - Nghị định 168:2024/NĐ-CP). Mức phạt cho hành vi này là từ 400.000 đồng đến 600.000 đồng.
+3. **Gây tai nạn và không dừng lại**: Sau khi gây tai nạn, người điều khiển xe không dừng lại, không trợ giúp người bị nạn, và không trình báo với cơ quan có thẩm quyền, vi phạm quy định về xử lý sau tai nạn (Điều 7, Khoản 9, Điểm c - Nghị định 168:2024/NĐ-CP). Mức phạt cho hành vi này là từ 8.000.000 đồng đến 10.000.000 đồng.
+Các điều khoản không đề cập tới việc xử lý hành vi chửi bới người bị nạn.</t>
+  </si>
+  <si>
+    <t>Mng cho em hỏi tầm bao lâu có thông báo phạt nguôi trê app vậy ạ. Thấy luật để 10 ngày không biết thực tế là bao nhiêu em ở Trà Vinh.</t>
+  </si>
+  <si>
+    <t>Em bị tạm giam xe do không đội mũ và quên mang giấy tờ - đã kí biên bản
+-xe của em là mua bán chưa sang tên (có giấy đ ký gốc)- đã mất hợp đồng mua bán và mất liên lạc với chủ cũ
+Mọi người cho em hỏi , em đi đóng phạt thì có lấy đc xe hay ko ?
+có bắt buộc phải liên lạc với chủ cũ để chủ cũ lên đóng phạt mới lấy đc xe hay ko ?
+Mong mọi người trả lời , em xin cảm ơn</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời toàn bộ câu hỏi của bạn. Tuy nhiên, tôi có thể cung cấp một số thông tin liên quan như sau:
+1. Về việc không đội mũ bảo hiểm: Hành vi không đội mũ bảo hiểm khi điều khiển xe mô tô, xe máy có thể bị phạt tiền từ 400.000 đồng đến 600.000 đồng (Điều 7, Khoản 2, Điểm h - Nghị định 168:2024/NĐ-CP).
+2. Về việc không mang giấy tờ: Nếu bạn không xuất trình được giấy tờ cần thiết tại thời điểm kiểm tra, bạn có thể bị xử phạt hành chính. Tuy nhiên, nếu bạn xuất trình được các giấy tờ trong thời hạn hẹn đến giải quyết vụ việc vi phạm ghi trong biên bản, thì người có thẩm quyền có thể ra quyết định xử phạt về hành vi không mang theo giấy tờ (Điều 48, Khoản 3, Điểm b - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc bạn có cần liên lạc với chủ cũ để lấy xe hay không, cũng như không có thông tin về việc xử lý trong trường hợp xe chưa sang tên.</t>
+  </si>
+  <si>
+    <t>Các bác cho cháu hỏi là nay cháu bị công an bắt kh mũ và có bạn cháu kh mũ thì các chú công an kiểm tra vneid với xem bằng lái rồi cho cháu viết biên bản rồi cho cháu cầm về hẹn lên nộp phạt chứ không giữ giấy tờ gì và cho cháu cầm xe về ạ cho cả bạn cháu viết vậy thì phải nộp bao nhiêu tiền ạ cháu lần đầu bị như này cháu rất rối ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, bạn và bạn của bạn có thể bị phạt tiền từ 400.000 đồng đến 600.000 đồng mỗi người vì hành vi không đội mũ bảo hiểm hoặc đội mũ bảo hiểm không cài quai đúng quy cách khi điều khiển xe mô tô, xe máy tham gia giao thông trên đường bộ (Điều 7, Khoản 2, Điểm h - Nghị định 168:2024/NĐ-CP). Các điều khoản không đề cập tới việc xử lý giấy tờ hay quy trình cụ thể khi bị xử phạt.</t>
+  </si>
+  <si>
+    <t>Máy bác cho em hỏi bữa em bị bắt xe máy bị giam phương tiện hiện em đã đóng phạt rồi sao trên app vẫn hiện chưa xử phạt</t>
+  </si>
+  <si>
+    <t>các bác cho em hỏi bé nhà em chưa đủ 16 tuổi, em có mua cái xe Chaly tàu cũ, trên đk xe ghi thông tin 49cc. con đi học gần nhà nên chủ quan không đội mũ, không gương. và xe cũ qua nhiều đời chủ nên em cũng không đổi đăng ký. giờ con bị csgt vào trường bắt xe. em lên giải quyết nộp phạt thì cán bộ nhất quyết yêu cầu em cung cấp giấy mua bán xe. em thì ở Hà Nội, chủ xe Thái Bình, xe cũ quá ròi em chấp nhận để tịch thu xe và mong muốn giải quyết biên bản là nộp phạt theo quy định, nhưng cán bộ không giải quyết, em đã lên 3 lần rồi vẫn bắt em lấy giấy mua bán xe mới giải quyết. Bây giờ em nên làm sao ạ? cứ để biên bản vậy không giải quyết thì bé nhà em có ảnh hưởng gì về pháp luật không ạ ?</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, có một số thông tin liên quan đến tình huống của bạn:
+1. **Vi phạm không đội mũ bảo hiểm**: Bé nhà bạn không đội mũ bảo hiểm khi điều khiển xe, điều này có thể bị phạt tiền từ 400.000 đồng đến 600.000 đồng (Điều 7, Khoản 2, Điểm h - Nghị định 168:2024/NĐ-CP).
+2. **Vấn đề về giấy tờ xe**: Nếu xe không có chứng nhận đăng ký xe hoặc sử dụng chứng nhận đăng ký xe không do cơ quan có thẩm quyền cấp, không đúng số khung, số động cơ hoặc bị tẩy xóa mà không chứng minh được nguồn gốc xuất xứ của phương tiện, thì xe có thể bị tịch thu (Điều 14, Khoản 5, Điểm b - Nghị định 168:2024/NĐ-CP).
+3. **Yêu cầu giấy mua bán xe**: Các điều khoản không đề cập cụ thể tới việc yêu cầu giấy mua bán xe để giải quyết vi phạm. Tuy nhiên, việc chứng minh nguồn gốc xuất xứ của phương tiện là cần thiết để tránh bị tịch thu xe.
+4. **Ảnh hưởng pháp luật đối với bé**: Các điều khoản không đề cập tới việc bé nhà bạn có bị ảnh hưởng pháp luật gì nếu không giải quyết biên bản.
+Với tình huống hiện tại, bạn có thể cần tìm cách chứng minh nguồn gốc hợp pháp của xe để tránh việc bị tịch thu. Nếu không thể cung cấp giấy tờ cần thiết, việc xe bị tịch thu có thể xảy ra theo quy định.</t>
+  </si>
+  <si>
+    <t>Mn ơi xe đạp gắn trợ lực vào thì bao nhiêu tuổi đc đi vậy?</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời câu hỏi về độ tuổi được phép điều khiển xe đạp gắn trợ lực.</t>
+  </si>
+  <si>
+    <t>E chưa blx bị tai nạn do tông phải ng kia đi ngược chiều 2 bên thỏa thuận tình cảm thì e bị phạt bao tiền ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, nếu bạn điều khiển xe mô tô hai bánh có dung tích xi-lanh đến 125 cm3 hoặc có công suất động cơ điện đến 11 kW mà không có giấy phép lái xe, bạn sẽ bị phạt tiền từ 2.000.000 đồng đến 4.000.000 đồng (Điều 18, Khoản 5, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử lý tình huống tai nạn giao thông khi hai bên đã thỏa thuận tình cảm.</t>
+  </si>
+  <si>
+    <t>Chỗ em bây giờ học sinh cấp 2 chạy xe đạp điện cũng bị bắt nữa,phạt thì cao,không biết phải làm sao đây,nhà thì xa trường bố mẹ thì bận không chở đi học được</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc học sinh cấp 2 điều khiển xe đạp điện có thể bị xử phạt nếu vi phạm các quy tắc giao thông đường bộ. Cụ thể, các hành vi vi phạm có thể bị phạt tiền từ 100.000 đồng đến 200.000 đồng bao gồm:
+- Không đi bên phải theo chiều đi của mình, đi không đúng phần đường quy định (Điều 9, Khoản 1, Điểm a - Nghị định 168:2024/NĐ-CP).
+- Dừng xe đột ngột; chuyển hướng không báo hiệu trước (Điều 9, Khoản 1, Điểm b - Nghị định 168:2024/NĐ-CP).
+- Không chấp hành hiệu lệnh hoặc chỉ dẫn của biển báo hiệu, vạch kẻ đường (Điều 9, Khoản 1, Điểm c - Nghị định 168:2024/NĐ-CP).
+- Vượt bên phải trong các trường hợp không được phép (Điều 9, Khoản 1, Điểm d - Nghị định 168:2024/NĐ-CP).
+- Dừng xe, đỗ xe trên phần đường xe chạy ở đoạn đường ngoài đô thị nơi có lề đường (Điều 9, Khoản 1, Điểm đ - Nghị định 168:2024/NĐ-CP).
+- Chạy trong hầm đường bộ không bật đèn hoặc không có vật phát sáng báo hiệu (Điều 9, Khoản 1, Điểm e - Nghị định 168:2024/NĐ-CP).
+- Điều khiển xe đạp, xe đạp máy đi dàn hàng ngang từ 03 xe trở lên (Điều 9, Khoản 1, Điểm g - Nghị định 168:2024/NĐ-CP).
+- Sử dụng ô (dù), dùng tay cầm và sử dụng điện thoại hoặc các thiết bị điện tử khác khi điều khiển xe (Điều 9, Khoản 1, Điểm h - Nghị định 168:2024/NĐ-CP).
+- Điều khiển xe thô sơ trong thời gian từ 18 giờ ngày hôm trước đến 06 giờ ngày hôm sau không sử dụng đèn hoặc không có báo hiệu ở phía trước và phía sau xe (Điều 9, Khoản 1, Điểm i - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc học sinh cấp 2 có được phép điều khiển xe đạp điện hay không, cũng như không nêu rõ mức phạt cụ thể cho việc điều khiển xe đạp điện khi chưa đủ tuổi.</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi, em điều khiển xe máy điện chưa đăng kí. Thì CSGT phạt cả việc xe không có đăng kí kèm không gắn biển số là 2 lỗi. Nhưng chưa đăng kí thì sao có biển số được ạ. Trường hợp này em nên làm như thế nào ạ</t>
+  </si>
+  <si>
+    <t>Mấy bác cho e hỏi e bỏ cây sắt trong cốp xe rồi bị CA giao thông kiểm tra và phạt 15tr e thấy vô lý quá e k đóng , rồi sau này có sao k các bác , với lại thấy lãi 0,05 một ngày e sợ quá ạ. Có bác nào rành cho e xin góp ý chút ạ , e cảm ơn</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời câu hỏi này. Không có điều khoản nào trong danh sách cung cấp đề cập đến việc xử phạt liên quan đến việc mang theo cây sắt trong cốp xe hoặc mức phạt 15 triệu đồng.</t>
+  </si>
+  <si>
+    <t>Cho e hỏi e gây tngt bị giam xe mình tự đi lấy xe hay đợi gọi mới được lấy ạ</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đề cập tới việc bạn cần tự đi lấy xe hay đợi gọi mới được lấy xe sau khi bị giam giữ do gây tai nạn giao thông.</t>
+  </si>
+  <si>
+    <t>Đêm hôm qua em đi được 1 đoạn bị hình sự rình bắt xe về đồn bị quên giấy tờ xe và không có bằng lái xe họ nói nào có bằng lái xe hay có tiền hẳn nói chuyện sử lý sao vậy mọi người
+Em mới 22 tuổi mà chưa có bằng lái xe ạ họ nói không có bằng phạt gần chục triệu nghe khổ quá ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, nếu bạn điều khiển xe mô tô hai bánh có dung tích xi-lanh đến 125 cm3 mà không có giấy phép lái xe, bạn có thể bị phạt tiền từ 2.000.000 đồng đến 4.000.000 đồng (Điều 18, Khoản 5, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử lý khi quên giấy tờ xe hoặc yêu cầu "có tiền hẳn nói chuyện".</t>
+  </si>
+  <si>
+    <t>Dạ cho e hỏi là e láy xe gặp tai nạn và e k có bằng lái nhưng e chạy đúng và xe chính chủ thì phạt bao nhiu ạ ( cứu e)</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc bạn điều khiển xe mà không có giấy phép lái xe là hành vi bị nghiêm cấm (Điều 9, Khoản 1 - Luật số: 36/2024/QH15). 
+Về mức phạt, nếu bạn điều khiển xe ô tô hoặc các loại xe tương tự mà không có giấy phép lái xe, bạn sẽ bị phạt tiền từ 18.000.000 đồng đến 20.000.000 đồng (Điều 18, Khoản 9, Điểm b - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc bạn chạy đúng hay xe chính chủ có ảnh hưởng gì đến mức phạt hay không.</t>
+  </si>
+  <si>
+    <t>M.n trong nhóm chia sẽ giúp em với ạ. Giờ em phải làm sao đây? 
+Tết 2024 em có vi phạm giao thông về vựơt quá tốc độ ở tỉnh Đồng Nai, công an tịch thu bằng và đưa biên bản cho em, có kèm sđt bưu điện để đóng phạt ( vì em ở SG). Nhưng thời điểm đó em gặp khó khăn kinh tế do thất nghiệp, nên không đóng phạt đựơc. Trong năm đó đt em bị hư, mất luôn sdt bưu điện, và sdt. Tới hiện tại thì kinh tế em đã tốt hơn 1 chút, nên em muốn xin nộp phạt và lấy lại gplx, nhưng tra cứu thì không hiện thông tin nữa. Em rối quá, nhờ cả nhà giúp đỡ ạ</t>
+  </si>
+  <si>
+    <t>Mọi người ai có văn bản tường trình để nhận lại bằng lái bị tước đó vi phạm nồng độ cồn kh ạ ? E kh biết ghi và mấy a công an giao thông cũng kh hướng dẫn luôn ạ</t>
+  </si>
+  <si>
+    <t>Em bị vi phạm nồng độ cồn từ tháng 10/2024. Bị giữ GPLX 11 tháng tới tháng 9/2025 
+Đến ngày hẹn đã đến phòng CSGT để nhập giấy phép Lx mà đến hiện tại hơn 1 tháng sau khi đến yêu cầu nhận lại mà chưa nhận được thì phải làm sao ạ</t>
+  </si>
+  <si>
+    <t>Cho e hỏi e vi phạm giao thông (đi vào làn brt) xe máy điện không giấy tờ không gương không biển số bị ký biên bản r thì bị phạt bao nhiêu ạ.</t>
+  </si>
+  <si>
+    <t>em bị phạt số tiền quá nhiều hơn giá trị xe giờ em quyết định bỏ xe nhưng em nghe nếu k đóng sẽ cộng lãi 0.05% ngày.Cái này là thiệt k dạ anh chị.Em cảm ơn</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đề cập tới việc tính lãi suất 0.05% mỗi ngày nếu không đóng phạt.</t>
+  </si>
+  <si>
+    <t>anh em rành luật cho e hỏi, trước đó e vi phạm lỗi quá tốc độ mà chưa đóng phạt nên bị giam bằng trên vneid, xong sau e bị bắt lỗi nồng độ cồn kịch khung tiếp, thì bị phạt tổng bao nhiêu ạ? và có bị tính lỗi ko có bằng lái ko ạ</t>
+  </si>
+  <si>
+    <t>Ai hiểu luật cho em hỏi với Lúc bị bắt khai tuổi giả h đi lấy xe đưa cccd có tuổi thật người ta có cho lấy xe ko ạ</t>
+  </si>
+  <si>
+    <t>E bị phạt tội không chấp hành đèn giao thông thì bị phạt tầm bao nhiêu tiền vậy moi người oi</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời câu hỏi này, vì không có điều khoản nào đề cập đến mức phạt cho hành vi không chấp hành đèn giao thông.</t>
+  </si>
+  <si>
+    <t>Mng cho em hỏi em mới thi đậu bằng C1 hôm 13/10 , mà trước đó tầm 5 tháng em có bị giam bằng A1 do quá tốc độ . Mng cho e hỏi là e bị như v thì có ảnh hưởng gì tới thời gian cấp bằng và cấp số gplx trên vneid k ạ ? E vẫn đc thi và đậu bằng C1 ngày 13/10</t>
+  </si>
+  <si>
+    <t>Dạ cho em hỏi em vừa bị bắt vì đi ngược chiều, anh CS bảo là đi ngc chiều bị phạt 5tr vs trừ điểm, rồi anh ấy có lấy BLX của em và ghi lại vào giấy nhớ rồi trả lại luôn, rồi bảo em về đi, như thế em có bị phạt không ạ, và em phải ktra xem mình có bị phạt không ở đâu ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc đi ngược chiều có thể bị xử phạt như sau:
+1. Nếu bạn điều khiển xe ô tô hoặc xe tương tự và đi ngược chiều của đường một chiều hoặc trên đường có biển “Cấm đi ngược chiều”, bạn có thể bị phạt tiền từ 18.000.000 đồng đến 20.000.000 đồng (Điều 6, Khoản 9, Điểm d - Nghị định 168:2024/NĐ-CP).
+2. Nếu bạn điều khiển xe đi ngược chiều trên đường cao tốc, mức phạt sẽ cao hơn, từ 30.000.000 đồng đến 40.000.000 đồng (Điều 6, Khoản 11, Điểm đ - Nghị định 168:2024/NĐ-CP).
+Về việc kiểm tra xem bạn có bị phạt hay không, các điều khoản không đề cập tới cách thức kiểm tra tình trạng xử phạt. Tuy nhiên, thông thường, bạn có thể kiểm tra thông tin xử phạt qua các kênh thông tin của cơ quan công an giao thông hoặc qua các cổng thông tin điện tử của cơ quan nhà nước có thẩm quyền.</t>
+  </si>
+  <si>
+    <t>Mn cho em hỏi. Em bán xe 70250 cho cửa hàng 2 năm rồi. Mà chưa có ai rút sang tên. Lỡ người mua mà vi phạm là toang luôn. Có cách nào ko mn. Em cám ơn</t>
+  </si>
+  <si>
+    <t>Dạ cho em hỏi em vừa bị bắt vì rẽ trái ngay biển báo cấm, CS bảo là bị phạt 700 nhưng không bị trừ điểm vneid, rồi CS có giữ BLX của em và gửi em 1 biên bản để em giữ, rồi bảo đến ngày hẹn tuần sau thì lên đội CSGT nộp phạt và lấy lại BLX. Khi về em tra trên DVC thì không thấy gì cả. Với em thắc mắc là mình lên nộp phạt trực tiếp ở địa chỉ đội CSGT đó được đúng không ạ hay phải ra ngân hàng hay khi bạc nhà nuớc đóng và em sau khi đóng xong em có được trả BLX liền không hay đợi nữa ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc bạn điều khiển xe rẽ trái tại nơi có biển báo hiệu cấm rẽ trái là hành vi vi phạm quy tắc giao thông đường bộ. Mức phạt tiền cho hành vi này là từ 1.000.000 đồng đến 2.000.000 đồng nếu bạn điều khiển xe máy chuyên dùng (Điều 8, Khoản 4, Điểm d - Nghị định 168:2024/NĐ-CP) và từ 2.000.000 đồng đến 3.000.000 đồng nếu bạn điều khiển xe ô tô hoặc các loại xe tương tự (Điều 6, Khoản 4, Điểm k - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc bạn có thể nộp phạt trực tiếp tại địa chỉ đội CSGT hay phải ra ngân hàng hoặc kho bạc nhà nước để đóng phạt. Cũng không có thông tin về việc bạn có được trả lại giấy phép lái xe ngay sau khi đóng phạt hay không.</t>
+  </si>
+  <si>
+    <t>mọi người ơi cho e hỏi đi xe dưới 50cc (49) có cần bằng lái không ạ
+mẹ e đọc được mấy bài bảo giờ ra đường xe nào cũng phải có bằng rồi gọi hỏi chỗ thi bằng là xe dưới 50cc có cần bằng không thì họ bảo có</t>
+  </si>
+  <si>
+    <t>Em bị thổi nồng độ cồn xe máy bị tước bằng 23 tháng , vậy có được thi sát hạch bằng ô tô không ạ , em mấy tháng nữa thi rồi huhu</t>
+  </si>
+  <si>
+    <t>Chả là em đi xe máy điện và bị bắt lỗi điều khiển xe k biển số và điều khiển xe k có chứng nhận đăng kí xe. Nghe nói phạt nhiều lắm ạ, em đang muốn hỏi nếu em bỏ xe có sao k ạ? Có ng kêu CAGT có thông tin của mk rồi mk vi phạm thế này mà k lấy xe sau mk mua xe khác hoặc liên quan giấy tờ mua bán gì về sau rất khó có phải k ạ?</t>
+  </si>
+  <si>
+    <t>mng ơi, em và bạn em lớp 12. Nó đi xe 110 và không đội mũ, em có đội mũ. Hôm nay xe hỏng em đi nhờ cùng nó, xog đến cổng trường em xuống, đi được 3 4 bước rồi thì công an bắt nó. Nó bảo lên đó công an hỏi cả tên vs tủoo của em thì em có bị sao không ạ</t>
+  </si>
+  <si>
+    <t>Mọi người cho hỏi mình bị bắt nồng độ cồn dưới 0,25 thì phạt bao nhiêu , trong biên bản hẹn 28/10 mà mình có thể đóng trước để lấy xe ra không ạ xe máy</t>
+  </si>
+  <si>
+    <t>Theo quy định tại Nghị định 168:2024/NĐ-CP, nếu bạn điều khiển xe máy mà trong máu hoặc hơi thở có nồng độ cồn chưa vượt quá 0,25 miligam/1 lít khí thở, bạn sẽ bị phạt tiền từ 2.000.000 đồng đến 3.000.000 đồng (Điều 7, Khoản 6, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc bạn có thể đóng phạt trước để lấy xe ra hay không.</t>
+  </si>
+  <si>
+    <t>ACE cho e hỏi tí xe máy chạy vào lane oto thì phạt bao nhiu vậy ạ. Cho mượn xe giờ lãnh đủ luôn. Thank ace nhìu.</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc điều khiển xe máy chạy vào làn đường dành cho ô tô có thể bị coi là vi phạm quy tắc giao thông đường bộ, cụ thể là không chấp hành hiệu lệnh, chỉ dẫn của biển báo hiệu, vạch kẻ đường. Hành vi này có thể bị phạt tiền từ 200.000 đồng đến 400.000 đồng (Điều 7, Khoản 1, Điểm a - Nghị định 168:2024/NĐ-CP). Các điều khoản không đề cập cụ thể đến việc xử phạt người cho mượn xe.</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi lỗi vi phạm lấn làn xe máy là bao nhiêu vậy nay em đóng là 2tr6 mà về lên mạng tra cứu lại thù có từ 600-800k. Em hoang mang quá</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đề cập cụ thể đến mức phạt cho hành vi vi phạm lấn làn xe máy. Tuy nhiên, có một số điều khoản liên quan đến các hành vi vi phạm khác của người điều khiển xe mô tô, xe gắn máy với mức phạt từ 200.000 đồng đến 400.000 đồng (Điều 7, Khoản 1, Điểm a-e - Nghị định 168:2024/NĐ-CP). 
+Vì vậy, không có căn cứ từ các điều khoản cung cấp để xác định mức phạt 2.600.000 đồng cho lỗi lấn làn xe máy.</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi em bị bắt không gplx và xe em mua củ lâu rồi không phải em đứng tên, nhưng lập biên bản thông tin là của em , nhưng phạt nặng quá em không đóng phạt có sao ạ</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, việc bạn điều khiển xe mà không có giấy phép lái xe có thể bị phạt tiền từ 2.000.000 đồng đến 4.000.000 đồng (Điều 18, Khoản 5, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử lý khi bạn không đóng phạt. Tuy nhiên, thông thường, việc không đóng phạt có thể dẫn đến các biện pháp cưỡng chế thi hành quyết định xử phạt theo quy định của pháp luật.</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi em đỗ xe máy mua hoa quả và bị xử phạt. Mức phạt là 400k đến 600k . Vậy trường hợp của em bị phạt cụ thể là bao nhiêu ạ</t>
+  </si>
+  <si>
+    <t>Theo các điều khoản được cung cấp, việc bạn đỗ xe máy để mua hoa quả có thể bị xử phạt từ 400.000 đồng đến 600.000 đồng nếu vi phạm một trong các hành vi sau:
+1. Dừng xe, đỗ xe trên phần đường xe chạy ở đoạn đường ngoài đô thị nơi có lề đường (Điều 7, Khoản 2, Điểm a - Nghị định 168:2024/NĐ-CP).
+2. Dừng xe, đỗ xe ở lòng đường gây cản trở giao thông; tụ tập từ 03 xe trở lên ở lòng đường, trong hầm đường bộ; đỗ, để xe ở lòng đường, vỉa hè trái phép (Điều 7, Khoản 2, Điểm d - Nghị định 168:2024/NĐ-CP).
+3. Dừng xe, đỗ xe trên điểm đón, trả khách, nơi đường bộ giao nhau, trên phần đường dành cho người đi bộ qua đường; dừng xe nơi có biển “Cấm dừng xe và đỗ xe”; đỗ xe tại nơi có biển “Cấm đỗ xe” hoặc biển “Cấm dừng xe và đỗ xe”; không tuân thủ các quy định về dừng xe, đỗ xe tại nơi đường bộ giao nhau cùng mức với đường sắt; dừng xe, đỗ xe trong phạm vi hành lang an toàn giao thông đường sắt (Điều 7, Khoản 2, Điểm e - Nghị định 168:2024/NĐ-CP).
+Mức phạt cụ thể trong khoảng từ 400.000 đồng đến 600.000 đồng sẽ do cơ quan có thẩm quyền quyết định dựa trên tình huống cụ thể của bạn. Các điều khoản không đề cập tới việc xác định mức phạt cụ thể trong khoảng này.</t>
+  </si>
+  <si>
+    <t>Bằng B2 của em sắp hết hạn . Nhưng em tra trên hệ thống vnetraffic có 1 xe máy cũ đứng tên em đã bán từ rất lâu hơn 10 năm , không còn giữ giấy tờ mua bán , đang dính phạt nồng độ cồn kịch khung , không xuất trình giấy tờ , lỗi giao xe cho người không đủ điều kiện . Vậy cho em hỏi giờ mình phải tự lên đóng phạt hay làm đơn trình bày mới đổi được giấy phép ô tô B2 lên C1 ạ . Em cảm ơn</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời toàn bộ câu hỏi của bạn. Tuy nhiên, tôi có thể cung cấp một số thông tin liên quan như sau:
+1. Về việc xử phạt hành vi không xuất trình giấy tờ: Nếu trong thời hạn hẹn đến giải quyết vụ việc vi phạm ghi trong biên bản vi phạm hành chính, người vi phạm xuất trình được các giấy tờ hoặc thông tin của các giấy tờ được tích hợp trong tài khoản định danh điện tử theo quy định, thì người có thẩm quyền không ra quyết định xử phạt vi phạm hành chính đối với hành vi vi phạm không có giấy tờ, không mang theo giấy tờ và không xử phạt đối với chủ phương tiện (Điều 48, Khoản 3, Điểm c - Nghị định 168:2024/NĐ-CP).
+2. Về hành vi giao xe cho người không đủ điều kiện: Chủ xe mô tô, xe gắn máy và các loại xe tương tự xe mô tô, các loại xe tương tự xe gắn máy có thể bị phạt 20.000.000 đồng nếu thực hiện hành vi vi phạm giao xe hoặc để cho người không đủ điều kiện điều khiển xe tham gia giao thông (Điều 32, Khoản 20 - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc bạn có cần tự lên đóng phạt hay làm đơn trình bày để đổi giấy phép lái xe từ B2 lên C1.</t>
+  </si>
+  <si>
+    <t>Em chào tất cả anh chị trong nhóm anh chị cho em hỏi chút với ạ hnay là thế này cháu em năm nay học lớp 12 sáng nay xe chaus hỏng và chaus hỏi mượn xe em em ko cho mượn nhưng chaus vẫn cố tình lấy xs đi và bị công an đội 10 ở Hà Nội bắt và lập biên bản hội hẹn 28 tháng này ra lấy em có cần phải đi thép để giải quyết ko ạ hay chỉ cần mẹ hoặc bố đi là đc ạ xe em chính chủ ạ</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đề cập tới việc ai cần phải có mặt để giải quyết khi xe bị lập biên bản vi phạm giao thông. Do đó, tôi không thể xác định liệu bạn hay bố mẹ của cháu cần phải có mặt để giải quyết vấn đề này.</t>
+  </si>
+  <si>
+    <t>E có bằng A xe máy tới 175cc, thì khi ra đường cần thêm các giấy tờ nào khác ngoài cccd vs bằng lái xe + cà vẹt xe( của người thân cmdc ko ạ ) để ko bị pikachu dịnh lại đòi tiền vậy ạ</t>
+  </si>
+  <si>
+    <t>Khi điều khiển xe máy có dung tích xi-lanh tới 175cc, ngoài căn cước công dân (CCCD) và giấy phép lái xe, bạn cần mang theo các giấy tờ sau để tránh bị xử phạt:
+1. Chứng nhận đăng ký xe (cà vẹt xe). Nếu xe thuộc sở hữu của người khác, bạn cần có bản sao chứng nhận đăng ký xe có chứng thực kèm theo bản gốc giấy biên nhận còn hiệu lực của tổ chức tín dụng, chi nhánh ngân hàng nước ngoài trong trường hợp tổ chức tín dụng, chi nhánh ngân hàng nước ngoài giữ bản gốc chứng nhận đăng ký xe (Điều 48, Khoản 3, Điểm b - Nghị định 168:2024/NĐ-CP).
+2. Giấy chứng nhận kiểm định an toàn kỹ thuật và bảo vệ môi trường (nếu có yêu cầu đối với loại xe bạn điều khiển) (Điều 48, Khoản 3, Điểm b - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc cần mang theo giấy tờ nào khác ngoài những giấy tờ đã nêu trên.</t>
+  </si>
+  <si>
+    <t>Dạ các bác cho em hỏi thăm ạ, năm ngoái em có vi phạm giao thông vì chở hàng cồng kềnh xe máy nên bị giam gplx, sau khi em chuyển nhà thì làm thất lạc biên bản thời gian gần đây mới tìm ra được, thì cho em hỏi là em lên nộp phạt để lấy lại gplx được không và sẽ bị phạt như thế nào ạ. Em cám ơn ạ</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi em vừa bị trộm túi trong đó có giấy tờ gốc xe máy với bằng lái xe gồm đt tiền mặt thì. Cho em hỏi mất 2 thứ đó thì h mình có thể xin làm lại bằng lái xe ko ạcho e hỏi xíu là xe máy bị 141 bắt giữ xe trên phường thì tầm bao lâu dc trả xe ạ</t>
+  </si>
+  <si>
+    <t>Các bạn cho mình hỏi, mình cho bạn mượn xe bị bắt và phạt 3 lỗi là chạy quá tốc độ từ 5-10km, không có giấy phép lái xe, không có chứng nhận đăng ký xe (lỗi trên giấy ghi tên bạn ấy) thì chỉ cần bạn ấy lên nộp phạt là được lấy xe về hay em phải cùng lên ạ, có phải là phạt cả em vì lỗi giao xe cho người không đủ điều kiện lái xe (không có bằng lái xe) không ạ.</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, có thể trả lời các khía cạnh của câu hỏi như sau:
+1. **Về việc bạn của bạn bị phạt**:
+   - Bạn của bạn bị phạt vì điều khiển xe chạy quá tốc độ quy định từ 5 km/h đến dưới 10 km/h với mức phạt từ 400.000 đồng đến 600.000 đồng (Điều 7, Khoản 2, Điểm b - Nghị định 168:2024/NĐ-CP).
+   - Bạn của bạn cũng bị phạt vì không có giấy phép lái xe với mức phạt từ 2.000.000 đồng đến 4.000.000 đồng (Điều 18, Khoản 5, Điểm a - Nghị định 168:2024/NĐ-CP).
+2. **Về việc không có chứng nhận đăng ký xe**:
+   - Nếu không có chứng nhận đăng ký xe, phương tiện có thể bị tịch thu nếu không chứng minh được nguồn gốc xuất xứ của phương tiện (Điều 14, Khoản 5, Điểm b - Nghị định 168:2024/NĐ-CP).
+3. **Về trách nhiệm của bạn (chủ xe)**:
+   - Các điều khoản không đề cập cụ thể đến việc xử phạt chủ xe khi giao xe cho người không có giấy phép lái xe trong trường hợp này. Tuy nhiên, nếu có quy định khác liên quan đến việc giao xe cho người không đủ điều kiện, bạn có thể bị xử phạt. Các điều khoản cung cấp không đủ căn cứ để xác định rõ ràng về việc này.
+4. **Về việc lấy xe về**:
+   - Các điều khoản không đề cập cụ thể đến quy trình lấy xe về sau khi bị xử phạt. Thông thường, người vi phạm cần hoàn thành việc nộp phạt và thực hiện các thủ tục cần thiết theo quy định của cơ quan chức năng để lấy xe về.
+Tóm lại, bạn của bạn cần nộp phạt cho các lỗi vi phạm đã nêu. Về việc bạn có cần lên cùng hay không, và việc bạn có bị phạt vì giao xe cho người không đủ điều kiện hay không, các điều khoản không cung cấp đủ thông tin để trả lời rõ ràng.</t>
+  </si>
+  <si>
+    <t>Em là tân sinh viên năm nhất mới lên do tay lái chưa vững và không quen đường nên em luôn đi chậm và chủ động nhường khi tham gia giao thông chứ không chạy vội. Tối hôm qua khi đang quẹo cua, trước mặt em là xe container đang quay đầu nên em chủ động nhường đợi xe quay đầu xong mới vượt lên. Lúc đang nhường thì em nghe tiếng còi xe ở đằng sau, quay ra thì thấy một chiếc xe ô tô, khoảng hai giây sau khi xe ô tô bóp 1 tiếng kèn duy nhất thì em nghe tiếng va chạm sau đuôi xe, chiếc xe ô tô trắng kia vừa tông em ngay giữa đường quốc lộ. Là con gái, lúc đó trời tối lại một thân một mình ở chỗ lạ nên em rất sợ, tài xế ô tô hạ cửa kính xe xuống nói gì đó em nghe không rõ rồi xe đó đi tiếp như không có chuyện gì, do hoảng quá nên em tấp vào lề kiểm tra xe, cũng may là người và xe không sao. Không biết bác tài có cố ý hay chỉ vô tình quẹt phải xe em nhưng trường hợp vừa rồi làm em rất sợ, em không biết sau này chuyện gì sẽ còn sảy ra khi tham gia giao thông nhưng hiện tại em cảm thấy không an toàn khi chạy trên đường nữa. Em cũng muốn lên đây để chia sẻ câu chuyện của mình thôi, chúc mọi người một ngày tốt lành.</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, hành vi của tài xế ô tô có thể vi phạm các quy định sau:
+1. Nếu tài xế ô tô gây tai nạn giao thông mà không dừng ngay phương tiện, không giữ nguyên hiện trường, không trợ giúp người bị nạn, không ở lại hiện trường hoặc không đến trình báo ngay với cơ quan công an, Ủy ban nhân dân nơi gần nhất, thì có thể bị phạt tiền từ 16.000.000 đồng đến 18.000.000 đồng (Điều 6, Khoản 8 - Nghị định 168:2024/NĐ-CP).
+2. Nếu tài xế ô tô điều khiển xe không quan sát, giảm tốc độ hoặc dừng lại để bảo đảm an toàn theo quy định mà gây tai nạn giao thông, thì có thể bị phạt tiền từ 20.000.000 đồng đến 22.000.000 đồng (Điều 6, Khoản 10, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử lý tình huống khi bạn cảm thấy không an toàn khi tham gia giao thông.</t>
+  </si>
+  <si>
+    <t>cho em hỏi em có không may bị bắt xe với 2 lỗi là không mang theo giấy tờ xe và không bằng (xe không phải tên mình mà tên người trong gia đình) thì khi đi nộp phạt cần nộp bao nhiêu và có yêu cầu chủ xe đến không ạ</t>
+  </si>
+  <si>
+    <t>Dựa trên các điều khoản được cung cấp, bạn có hai lỗi vi phạm:
+1. Không mang theo giấy tờ xe:
+   - Nếu bạn xuất trình được các giấy tờ trong thời hạn hẹn đến giải quyết vụ việc vi phạm ghi trong biên bản vi phạm hành chính, bạn sẽ bị xử phạt về hành vi không mang theo giấy tờ, nhưng không có thông tin cụ thể về mức phạt trong các điều khoản được cung cấp (Điều 48, Khoản 3, Điểm b - Nghị định 168:2024/NĐ-CP).
+2. Không có giấy phép lái xe:
+   - Bạn sẽ bị phạt tiền từ 2.000.000 đồng đến 4.000.000 đồng nếu điều khiển xe mô tô hai bánh có dung tích xi-lanh đến 125 cm3 mà không có giấy phép lái xe (Điều 18, Khoản 5, Điểm a - Nghị định 168:2024/NĐ-CP).
+Về việc có cần chủ xe đến khi nộp phạt hay không, các điều khoản không đề cập tới việc này.</t>
+  </si>
+  <si>
+    <t>dạ cả nhà cho e hỏi chút ạ . em rẽ phải quên xi nhan bị bắt trong đường khu công nghiệp. đồng chí lập biên bản cho em k ghi rõ họ tên ạ. và lúc bảo e phải nộp phạt 700. đóng tại chỗ hay đóng cho kho bạc cũng giữ bằng lái xe. mà đồng chí cho e sdt của bưu điện ạ, cứ bắt e gọi rồi đóng cho bưu điện thì bưu điện sẽ gửi giấy về nhà cho ạ. giờ e làm sao lấy bằng lái vì e sắp đi xa ạ.</t>
+  </si>
+  <si>
+    <t>Theo điều khoản được cung cấp, việc bạn rẽ phải mà không có tín hiệu báo hướng rẽ (xi nhan) là hành vi vi phạm quy tắc giao thông đường bộ và có thể bị phạt tiền từ 600.000 đồng đến 800.000 đồng (Điều 7, Khoản 3, Điểm a - Nghị định 168:2024/NĐ-CP).
+Các điều khoản không đề cập tới việc xử lý trường hợp biên bản không ghi rõ họ tên, cách thức nộp phạt qua bưu điện, hay cách lấy lại bằng lái xe. Bạn nên liên hệ trực tiếp với cơ quan công an giao thông đã lập biên bản để được hướng dẫn cụ thể về việc nộp phạt và lấy lại bằng lái xe.</t>
+  </si>
+  <si>
+    <t>Các bác cho e hỏi: vận tốc cho phép trên Map thông báo có chính xác không ah? Chứ Hn xe e báo 90, e chạy 82 mà các anh áo vàng thổi phạt bắn tốc độ e lỗi vượt quá 22km. Bảo đoạn đó 60km/h. E lên xe chạy tiếp 2km vẫn vận tốc cho phép 90km/h. E thắc mắc mà k biết cải, chấp nhận giấy phạt rõ nặng! Buồn quá cơ</t>
+  </si>
+  <si>
+    <t>Các điều khoản tìm được không đủ căn cứ để trả lời câu hỏi về độ chính xác của thông tin vận tốc trên bản đồ (Map) so với quy định thực tế. Các điều khoản chỉ đề cập đến mức phạt cho hành vi chạy quá tốc độ quy định, nhưng không có thông tin về việc xác định vận tốc cho phép trên các ứng dụng bản đồ.</t>
   </si>
 </sst>
 </file>
@@ -690,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.5" style="1" customWidth="1"/>
@@ -865,7 +1247,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="176" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" ht="176" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>35</v>
       </c>
@@ -873,7 +1255,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>36</v>
       </c>
@@ -881,7 +1263,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>38</v>
       </c>
@@ -889,7 +1271,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="112" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>39</v>
       </c>
@@ -897,7 +1279,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
@@ -905,7 +1287,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>43</v>
       </c>
@@ -913,7 +1295,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>45</v>
       </c>
@@ -921,7 +1303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="96" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>46</v>
       </c>
@@ -929,7 +1311,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="192" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" ht="192" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>48</v>
       </c>
@@ -937,7 +1319,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="144" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" ht="144" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>50</v>
       </c>
@@ -945,7 +1327,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>51</v>
       </c>
@@ -953,7 +1335,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="176" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" ht="176" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>52</v>
       </c>
@@ -961,7 +1343,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>54</v>
       </c>
@@ -969,7 +1351,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>56</v>
       </c>
@@ -977,7 +1359,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>58</v>
       </c>
@@ -985,7 +1367,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>59</v>
       </c>
@@ -993,7 +1375,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="160" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>60</v>
       </c>
@@ -1001,7 +1383,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="96" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>62</v>
       </c>
@@ -1009,7 +1391,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>63</v>
       </c>
@@ -1017,7 +1399,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>64</v>
       </c>
@@ -1025,7 +1407,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>65</v>
       </c>
@@ -1033,7 +1415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>66</v>
       </c>
@@ -1041,7 +1423,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>67</v>
       </c>
@@ -1049,7 +1431,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>68</v>
       </c>
@@ -1057,7 +1439,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>69</v>
       </c>
@@ -1065,7 +1447,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>70</v>
       </c>
@@ -1073,7 +1455,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="224" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" ht="224" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>71</v>
       </c>
@@ -1081,7 +1463,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>73</v>
       </c>
@@ -1089,7 +1471,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="112" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>75</v>
       </c>
@@ -1097,7 +1479,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>77</v>
       </c>
@@ -1105,7 +1487,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>79</v>
       </c>
@@ -1113,7 +1495,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>80</v>
       </c>
@@ -1121,7 +1503,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>81</v>
       </c>
@@ -1129,7 +1511,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>83</v>
       </c>
@@ -1137,7 +1519,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>85</v>
       </c>
@@ -1145,7 +1527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>86</v>
       </c>
@@ -1153,7 +1535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="160" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" ht="160" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>87</v>
       </c>
@@ -1161,7 +1543,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>89</v>
       </c>
@@ -1169,7 +1551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>90</v>
       </c>
@@ -1177,12 +1559,484 @@
         <v>91</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="288" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" ht="288" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="208" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="112" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="96" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="176" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="224" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="288" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="256" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="224" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="320" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="96" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="144" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="128" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="208" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="144" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="112" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="112" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="272" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="272" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="96" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="192" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="272" x14ac:dyDescent="0.2">
+      <c r="A117" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" ht="224" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="112" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" ht="80" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update query processing outputs, refine evaluation docs, and add land use law datasets
</commit_message>
<xml_diff>
--- a/src/Query/output/batch_result.xlsx
+++ b/src/Query/output/batch_result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranhuuduc/Documents/dev/Rag_Graph_LawLaw/src/Query/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DA0D9B-4258-F142-A0D5-C4723096B530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5429E46B-DB64-AD46-9831-E853E8338F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1280" yWindow="-18960" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5920" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kết quả" sheetId="1" r:id="rId1"/>
@@ -1077,6 +1077,7 @@
   <cols>
     <col min="1" max="1" width="54.5" style="1" customWidth="1"/>
     <col min="2" max="2" width="81.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="76.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>